<commit_message>
add lean startup year budget
</commit_message>
<xml_diff>
--- a/KNOMO_Worldwide_Tech_and_Costs.xlsx
+++ b/KNOMO_Worldwide_Tech_and_Costs.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive overview" sheetId="1" r:id="Rdb84adb9a1834057"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech stack" sheetId="2" r:id="R64d9018848304441"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly costs" sheetId="3" r:id="R354f210cf1ae477a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch checklist" sheetId="4" r:id="Raef95a02bc044bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive overview" sheetId="1" r:id="Rdaf4fc331c274e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech stack" sheetId="2" r:id="Rd7c962d6515649a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly costs" sheetId="3" r:id="Rd90e279ae72d48b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch checklist" sheetId="4" r:id="Rbab4329245fd42e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup year" sheetId="5" r:id="Rf6929ab228c74ba1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -81,7 +82,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -118,6 +119,31 @@
         <x:fgColor rgb="FF8E3B52"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF29353C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDFEBF6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF44576D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFAAC7D8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF8E3B52"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -139,7 +165,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="38">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -208,6 +234,31 @@
     <x:xf numFmtId="200" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1922,4 +1973,488 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="40" t="str">
+        <x:v>KNOMO startup-year budget (lean plan)</x:v>
+      </x:c>
+      <x:c r="B1" s="40"/>
+      <x:c r="C1" s="40"/>
+      <x:c r="D1" s="40"/>
+      <x:c r="E1" s="40"/>
+      <x:c r="F1" s="40"/>
+      <x:c r="G1" s="40"/>
+      <x:c r="H1" s="40"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="43" t="str">
+        <x:v>Assumes a bootstrapped first year: founders cover product/engineering, use free tiers until usage proves demand, and pay only for production reliability and media. All amounts are INR (₹).</x:v>
+      </x:c>
+      <x:c r="B2" s="43"/>
+      <x:c r="C2" s="43"/>
+      <x:c r="D2" s="43"/>
+      <x:c r="E2" s="43"/>
+      <x:c r="F2" s="43"/>
+      <x:c r="G2" s="43"/>
+      <x:c r="H2" s="43"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="47" t="str">
+        <x:v>Budget line</x:v>
+      </x:c>
+      <x:c r="B4" s="47" t="str">
+        <x:v>Monthly ₹</x:v>
+      </x:c>
+      <x:c r="C4" s="47" t="str">
+        <x:v>Annual ₹</x:v>
+      </x:c>
+      <x:c r="D4" s="47" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>Startup assumption</x:v>
+      </x:c>
+      <x:c r="F4" s="47" t="str">
+        <x:v>Trigger to upgrade</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="14" t="str">
+        <x:v>Domain + DNS + email</x:v>
+      </x:c>
+      <x:c r="B5" s="20" t="n">
+        <x:v>1800</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="n">
+        <x:f>IF(D5="One-time",B5,B5*12)</x:f>
+        <x:v>21600</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E5" s="14" t="str">
+        <x:v>One domain, DNS, transactional email starter tier</x:v>
+      </x:c>
+      <x:c r="F5" s="14" t="str">
+        <x:v>Upgrade when email volume or team grows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="14" t="str">
+        <x:v>Frontend hosting/CDN</x:v>
+      </x:c>
+      <x:c r="B6" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C6" s="20" t="n">
+        <x:f>IF(D6="One-time",B6,B6*12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E6" s="14" t="str">
+        <x:v>Free static hosting/CDN tier</x:v>
+      </x:c>
+      <x:c r="F6" s="14" t="str">
+        <x:v>Paid tier after bandwidth/build limits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="14" t="str">
+        <x:v>API hosting</x:v>
+      </x:c>
+      <x:c r="B7" s="20" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="C7" s="20" t="n">
+        <x:f>IF(D7="One-time",B7,B7*12)</x:f>
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E7" s="14" t="str">
+        <x:v>One always-on production API instance</x:v>
+      </x:c>
+      <x:c r="F7" s="14" t="str">
+        <x:v>Add a second instance after uptime/load target is missed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="14" t="str">
+        <x:v>Managed database</x:v>
+      </x:c>
+      <x:c r="B8" s="20" t="n">
+        <x:v>3500</x:v>
+      </x:c>
+      <x:c r="C8" s="20" t="n">
+        <x:f>IF(D8="One-time",B8,B8*12)</x:f>
+        <x:v>42000</x:v>
+      </x:c>
+      <x:c r="D8" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E8" s="14" t="str">
+        <x:v>Small managed Postgres/MySQL with backups</x:v>
+      </x:c>
+      <x:c r="F8" s="14" t="str">
+        <x:v>Upgrade for storage, HA or replicas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="14" t="str">
+        <x:v>Object storage</x:v>
+      </x:c>
+      <x:c r="B9" s="20" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="n">
+        <x:f>IF(D9="One-time",B9,B9*12)</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="D9" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="str">
+        <x:v>R2/S3 for uploads; lifecycle-delete abandoned media</x:v>
+      </x:c>
+      <x:c r="F9" s="14" t="str">
+        <x:v>Add retention tiers after media library grows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="14" t="str">
+        <x:v>Video processing/delivery</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="n">
+        <x:f>IF(D10="One-time",B10,B10*12)</x:f>
+        <x:v>36000</x:v>
+      </x:c>
+      <x:c r="D10" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E10" s="14" t="str">
+        <x:v>Cap uploads and minutes; use managed video/CDN only where needed</x:v>
+      </x:c>
+      <x:c r="F10" s="14" t="str">
+        <x:v>Add transcoding workers as creator activity grows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="14" t="str">
+        <x:v>Realtime/cache/queue</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="n">
+        <x:f>IF(D11="One-time",B11,B11*12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E11" s="14" t="str">
+        <x:v>Start with DB polling; add Redis only when live traffic needs it</x:v>
+      </x:c>
+      <x:c r="F11" s="14" t="str">
+        <x:v>Introduce Redis/WebSockets at sustained concurrency</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="14" t="str">
+        <x:v>Monitoring/security</x:v>
+      </x:c>
+      <x:c r="B12" s="20" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="C12" s="20" t="n">
+        <x:f>IF(D12="One-time",B12,B12*12)</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="D12" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E12" s="14" t="str">
+        <x:v>Free monitoring plus paid error tracking/WAF allowance</x:v>
+      </x:c>
+      <x:c r="F12" s="14" t="str">
+        <x:v>Upgrade after incident volume or compliance need</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="14" t="str">
+        <x:v>Backups/DR</x:v>
+      </x:c>
+      <x:c r="B13" s="20" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C13" s="20" t="n">
+        <x:f>IF(D13="One-time",B13,B13*12)</x:f>
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="str">
+        <x:v>Automated DB backup plus monthly restore drill</x:v>
+      </x:c>
+      <x:c r="F13" s="14" t="str">
+        <x:v>Add cross-region copies before larger launch</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="14" t="str">
+        <x:v>Support/moderation tools</x:v>
+      </x:c>
+      <x:c r="B14" s="20" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C14" s="20" t="n">
+        <x:f>IF(D14="One-time",B14,B14*12)</x:f>
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E14" s="14" t="str">
+        <x:v>Founder-led support and moderation</x:v>
+      </x:c>
+      <x:c r="F14" s="14" t="str">
+        <x:v>Hire part-time support after response SLA slips</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="14" t="str">
+        <x:v>Founder/contractor cash budget</x:v>
+      </x:c>
+      <x:c r="B15" s="20" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="C15" s="20" t="n">
+        <x:f>IF(D15="One-time",B15,B15*12)</x:f>
+        <x:v>300000</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="str">
+        <x:v>Small monthly allowance for design, QA, legal or infra help</x:v>
+      </x:c>
+      <x:c r="F15" s="14" t="str">
+        <x:v>Increase after revenue/funding milestone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="14" t="str">
+        <x:v>Company/legal/privacy setup</x:v>
+      </x:c>
+      <x:c r="B16" s="20" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="n">
+        <x:f>IF(D16="One-time",B16,B16*12)</x:f>
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="str">
+        <x:v>Terms, privacy, company/admin setup and basic review</x:v>
+      </x:c>
+      <x:c r="F16" s="14" t="str">
+        <x:v>Repeat only for major jurisdictions or fundraising</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="14" t="str">
+        <x:v>Production migration + launch hardening</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="n">
+        <x:v>75000</x:v>
+      </x:c>
+      <x:c r="C17" s="20" t="n">
+        <x:f>IF(D17="One-time",B17,B17*12)</x:f>
+        <x:v>75000</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E17" s="14" t="str">
+        <x:v>SQLite to managed DB, media storage, HTTPS, CI/CD</x:v>
+      </x:c>
+      <x:c r="F17" s="14" t="str">
+        <x:v>Repeat for major architecture change</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="14" t="str">
+        <x:v>Security/load testing</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="n">
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="n">
+        <x:f>IF(D18="One-time",B18,B18*12)</x:f>
+        <x:v>50000</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E18" s="14" t="str">
+        <x:v>Baseline test before public promotion</x:v>
+      </x:c>
+      <x:c r="F18" s="14" t="str">
+        <x:v>Repeat before major scale events</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="49" t="str">
+        <x:v>Startup recurring subtotal</x:v>
+      </x:c>
+      <x:c r="B19" s="52" t="n">
+        <x:f>SUM(B5:B18)</x:f>
+        <x:v>264800</x:v>
+      </x:c>
+      <x:c r="C19" s="52" t="n">
+        <x:f>SUM(C5:C18)</x:f>
+        <x:v>702600</x:v>
+      </x:c>
+      <x:c r="D19" s="49" t="str"/>
+      <x:c r="E19" s="49" t="str"/>
+      <x:c r="F19" s="49" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="49" t="str">
+        <x:v>One-time launch subtotal</x:v>
+      </x:c>
+      <x:c r="B20" s="52"/>
+      <x:c r="C20" s="52" t="n">
+        <x:f>SUMIF(D5:D18,"One-time",C5:C18)</x:f>
+        <x:v>225000</x:v>
+      </x:c>
+      <x:c r="D20" s="49" t="str"/>
+      <x:c r="E20" s="49" t="str"/>
+      <x:c r="F20" s="49" t="str"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="51" t="str">
+        <x:v>Total first-year startup cash need</x:v>
+      </x:c>
+      <x:c r="B21" s="53"/>
+      <x:c r="C21" s="53" t="n">
+        <x:f>C19+C20</x:f>
+        <x:v>927600</x:v>
+      </x:c>
+      <x:c r="D21" s="51" t="str"/>
+      <x:c r="E21" s="51" t="str"/>
+      <x:c r="F21" s="51" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="49" t="str">
+        <x:v>Startup operating rules</x:v>
+      </x:c>
+      <x:c r="B23" s="49"/>
+      <x:c r="C23" s="49"/>
+      <x:c r="D23" s="49"/>
+      <x:c r="E23" s="49"/>
+      <x:c r="F23" s="49"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="47" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="B24" s="47" t="str">
+        <x:v>Why it matters</x:v>
+      </x:c>
+      <x:c r="C24" s="47" t="str"/>
+      <x:c r="D24" s="47" t="str"/>
+      <x:c r="E24" s="47" t="str"/>
+      <x:c r="F24" s="47" t="str"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="14" t="str">
+        <x:v>Cap video duration and file size</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>Video is the largest variable cost; caps prevent surprise bills</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str"/>
+      <x:c r="D25" s="14" t="str"/>
+      <x:c r="E25" s="14" t="str"/>
+      <x:c r="F25" s="14" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="14" t="str">
+        <x:v>Use HTTPS from day one</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>Required for microphone access and protects login/session data</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str"/>
+      <x:c r="D26" s="14" t="str"/>
+      <x:c r="E26" s="14" t="str"/>
+      <x:c r="F26" s="14" t="str"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="14" t="str">
+        <x:v>Keep founder-led support/moderation</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>Preserves cash until usage and safety workload are proven</x:v>
+      </x:c>
+      <x:c r="C27" s="14" t="str"/>
+      <x:c r="D27" s="14" t="str"/>
+      <x:c r="E27" s="14" t="str"/>
+      <x:c r="F27" s="14" t="str"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="14" t="str">
+        <x:v>Review usage monthly</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>Upgrade only when measured traffic, storage or incidents justify it</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str"/>
+      <x:c r="D28" s="14" t="str"/>
+      <x:c r="E28" s="14" t="str"/>
+      <x:c r="F28" s="14" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>Keep 3 months runway</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>Recommended cash reserve: 3 × average monthly startup burn</x:v>
+      </x:c>
+      <x:c r="C29" t="str"/>
+      <x:c r="D29" t="str"/>
+      <x:c r="E29" t="str"/>
+      <x:c r="F29" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A23:F23"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
reduce startup budget assumptions
</commit_message>
<xml_diff>
--- a/KNOMO_Worldwide_Tech_and_Costs.xlsx
+++ b/KNOMO_Worldwide_Tech_and_Costs.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive overview" sheetId="1" r:id="Rdaf4fc331c274e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech stack" sheetId="2" r:id="Rd7c962d6515649a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly costs" sheetId="3" r:id="Rd90e279ae72d48b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch checklist" sheetId="4" r:id="Rbab4329245fd42e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup year" sheetId="5" r:id="Rf6929ab228c74ba1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive overview" sheetId="1" r:id="Rc388a1264da04478"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech stack" sheetId="2" r:id="R36a3277466ea4593"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly costs" sheetId="3" r:id="Rd510773e0ab94cef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch checklist" sheetId="4" r:id="R82c806b1ae10481a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup year" sheetId="5" r:id="R3b6a51d2982e4db5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup year - leaner" sheetId="6" r:id="Rb115121a755345ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -82,7 +83,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="13">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -144,6 +145,31 @@
         <x:fgColor rgb="FF8E3B52"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF29353C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDFEBF6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF44576D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFAAC7D8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF8E3B52"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -165,7 +191,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="55">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -259,6 +285,31 @@
     <x:xf numFmtId="200" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2457,4 +2508,488 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="57" t="str">
+        <x:v>KNOMO startup-year budget (lean plan)</x:v>
+      </x:c>
+      <x:c r="B1" s="57"/>
+      <x:c r="C1" s="57"/>
+      <x:c r="D1" s="57"/>
+      <x:c r="E1" s="57"/>
+      <x:c r="F1" s="57"/>
+      <x:c r="G1" s="57"/>
+      <x:c r="H1" s="57"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="60" t="str">
+        <x:v>Assumes a bootstrapped first year: founders cover product/engineering, use free tiers until usage proves demand, and pay only for production reliability and media. All amounts are INR (₹).</x:v>
+      </x:c>
+      <x:c r="B2" s="60"/>
+      <x:c r="C2" s="60"/>
+      <x:c r="D2" s="60"/>
+      <x:c r="E2" s="60"/>
+      <x:c r="F2" s="60"/>
+      <x:c r="G2" s="60"/>
+      <x:c r="H2" s="60"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="64" t="str">
+        <x:v>Budget line</x:v>
+      </x:c>
+      <x:c r="B4" s="64" t="str">
+        <x:v>Monthly ₹</x:v>
+      </x:c>
+      <x:c r="C4" s="64" t="str">
+        <x:v>Annual ₹</x:v>
+      </x:c>
+      <x:c r="D4" s="64" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="E4" s="64" t="str">
+        <x:v>Startup assumption</x:v>
+      </x:c>
+      <x:c r="F4" s="64" t="str">
+        <x:v>Trigger to upgrade</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="14" t="str">
+        <x:v>Domain + DNS + email</x:v>
+      </x:c>
+      <x:c r="B5" s="20" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="n">
+        <x:f>IF(D5="One-time",B5,B5*12)</x:f>
+        <x:v>10800</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E5" s="14" t="str">
+        <x:v>One domain and free/low-volume email tier</x:v>
+      </x:c>
+      <x:c r="F5" s="14" t="str">
+        <x:v>Upgrade when email volume or team grows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="14" t="str">
+        <x:v>Frontend hosting/CDN</x:v>
+      </x:c>
+      <x:c r="B6" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C6" s="20" t="n">
+        <x:f>IF(D6="One-time",B6,B6*12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E6" s="14" t="str">
+        <x:v>Free static hosting/CDN tier</x:v>
+      </x:c>
+      <x:c r="F6" s="14" t="str">
+        <x:v>Paid tier after bandwidth/build limits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="14" t="str">
+        <x:v>API hosting</x:v>
+      </x:c>
+      <x:c r="B7" s="20" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C7" s="20" t="n">
+        <x:f>IF(D7="One-time",B7,B7*12)</x:f>
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E7" s="14" t="str">
+        <x:v>Small production API tier; founders accept limited capacity</x:v>
+      </x:c>
+      <x:c r="F7" s="14" t="str">
+        <x:v>Add a second instance after uptime/load target is missed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="14" t="str">
+        <x:v>Managed database</x:v>
+      </x:c>
+      <x:c r="B8" s="20" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="C8" s="20" t="n">
+        <x:f>IF(D8="One-time",B8,B8*12)</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="D8" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E8" s="14" t="str">
+        <x:v>Small managed Postgres/MySQL with backups</x:v>
+      </x:c>
+      <x:c r="F8" s="14" t="str">
+        <x:v>Upgrade for storage, HA or replicas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="14" t="str">
+        <x:v>Object storage</x:v>
+      </x:c>
+      <x:c r="B9" s="20" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="n">
+        <x:f>IF(D9="One-time",B9,B9*12)</x:f>
+        <x:v>2400</x:v>
+      </x:c>
+      <x:c r="D9" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="str">
+        <x:v>Small R2/S3 bucket; delete abandoned media quickly</x:v>
+      </x:c>
+      <x:c r="F9" s="14" t="str">
+        <x:v>Add retention tiers after media library grows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="14" t="str">
+        <x:v>Video processing/delivery</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="n">
+        <x:f>IF(D10="One-time",B10,B10*12)</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="D10" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E10" s="14" t="str">
+        <x:v>Strict duration, size and monthly upload caps</x:v>
+      </x:c>
+      <x:c r="F10" s="14" t="str">
+        <x:v>Add transcoding workers as creator activity grows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="14" t="str">
+        <x:v>Realtime/cache/queue</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="n">
+        <x:f>IF(D11="One-time",B11,B11*12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E11" s="14" t="str">
+        <x:v>Start with DB polling; add Redis only when live traffic needs it</x:v>
+      </x:c>
+      <x:c r="F11" s="14" t="str">
+        <x:v>Introduce Redis/WebSockets at sustained concurrency</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="14" t="str">
+        <x:v>Monitoring/security</x:v>
+      </x:c>
+      <x:c r="B12" s="20" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C12" s="20" t="n">
+        <x:f>IF(D12="One-time",B12,B12*12)</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="D12" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E12" s="14" t="str">
+        <x:v>Free monitoring, logs and basic WAF rules</x:v>
+      </x:c>
+      <x:c r="F12" s="14" t="str">
+        <x:v>Upgrade after incident volume or compliance need</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="14" t="str">
+        <x:v>Backups/DR</x:v>
+      </x:c>
+      <x:c r="B13" s="20" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="C13" s="20" t="n">
+        <x:f>IF(D13="One-time",B13,B13*12)</x:f>
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="str">
+        <x:v>Automated DB backup plus monthly restore drill</x:v>
+      </x:c>
+      <x:c r="F13" s="14" t="str">
+        <x:v>Add cross-region copies before larger launch</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="14" t="str">
+        <x:v>Support/moderation tools</x:v>
+      </x:c>
+      <x:c r="B14" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" s="20" t="n">
+        <x:f>IF(D14="One-time",B14,B14*12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E14" s="14" t="str">
+        <x:v>Founder-led support and moderation using free tools</x:v>
+      </x:c>
+      <x:c r="F14" s="14" t="str">
+        <x:v>Hire part-time support after response SLA slips</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="14" t="str">
+        <x:v>Founder/contractor cash budget</x:v>
+      </x:c>
+      <x:c r="B15" s="20" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C15" s="20" t="n">
+        <x:f>IF(D15="One-time",B15,B15*12)</x:f>
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="str">
+        <x:v>No planned contractor spend; small emergency allowance</x:v>
+      </x:c>
+      <x:c r="F15" s="14" t="str">
+        <x:v>Increase after revenue/funding milestone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="14" t="str">
+        <x:v>Company/legal/privacy setup</x:v>
+      </x:c>
+      <x:c r="B16" s="20" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="n">
+        <x:f>IF(D16="One-time",B16,B16*12)</x:f>
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="str">
+        <x:v>Use templates plus one focused professional review</x:v>
+      </x:c>
+      <x:c r="F16" s="14" t="str">
+        <x:v>Repeat only for major jurisdictions or fundraising</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="14" t="str">
+        <x:v>Production migration + launch hardening</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="C17" s="20" t="n">
+        <x:f>IF(D17="One-time",B17,B17*12)</x:f>
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E17" s="14" t="str">
+        <x:v>DIY migration, HTTPS, CI/CD and storage setup</x:v>
+      </x:c>
+      <x:c r="F17" s="14" t="str">
+        <x:v>Repeat for major architecture change</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="14" t="str">
+        <x:v>Security/load testing</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="n">
+        <x:f>IF(D18="One-time",B18,B18*12)</x:f>
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E18" s="14" t="str">
+        <x:v>Basic checklist and low-cost test before promotion</x:v>
+      </x:c>
+      <x:c r="F18" s="14" t="str">
+        <x:v>Repeat before major scale events</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="66" t="str">
+        <x:v>Startup recurring subtotal</x:v>
+      </x:c>
+      <x:c r="B19" s="69" t="n">
+        <x:f>SUM(B5:B18)</x:f>
+        <x:v>75900</x:v>
+      </x:c>
+      <x:c r="C19" s="69" t="n">
+        <x:f>SUM(C5:C18)</x:f>
+        <x:v>195800</x:v>
+      </x:c>
+      <x:c r="D19" s="66" t="str"/>
+      <x:c r="E19" s="66" t="str"/>
+      <x:c r="F19" s="66" t="str"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="66" t="str">
+        <x:v>One-time launch subtotal</x:v>
+      </x:c>
+      <x:c r="B20" s="69"/>
+      <x:c r="C20" s="69" t="n">
+        <x:f>SUMIF(D5:D18,"One-time",C5:C18)</x:f>
+        <x:v>65000</x:v>
+      </x:c>
+      <x:c r="D20" s="66" t="str"/>
+      <x:c r="E20" s="66" t="str"/>
+      <x:c r="F20" s="66" t="str"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="68" t="str">
+        <x:v>Total first-year startup cash need</x:v>
+      </x:c>
+      <x:c r="B21" s="70"/>
+      <x:c r="C21" s="70" t="n">
+        <x:f>C19+C20</x:f>
+        <x:v>260800</x:v>
+      </x:c>
+      <x:c r="D21" s="68" t="str"/>
+      <x:c r="E21" s="68" t="str"/>
+      <x:c r="F21" s="68" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="66" t="str">
+        <x:v>Startup operating rules</x:v>
+      </x:c>
+      <x:c r="B23" s="66"/>
+      <x:c r="C23" s="66"/>
+      <x:c r="D23" s="66"/>
+      <x:c r="E23" s="66"/>
+      <x:c r="F23" s="66"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="64" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="B24" s="64" t="str">
+        <x:v>Why it matters</x:v>
+      </x:c>
+      <x:c r="C24" s="64" t="str"/>
+      <x:c r="D24" s="64" t="str"/>
+      <x:c r="E24" s="64" t="str"/>
+      <x:c r="F24" s="64" t="str"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="14" t="str">
+        <x:v>Cap video duration and file size</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>Video is the largest variable cost; caps prevent surprise bills</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str"/>
+      <x:c r="D25" s="14" t="str"/>
+      <x:c r="E25" s="14" t="str"/>
+      <x:c r="F25" s="14" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="14" t="str">
+        <x:v>Use HTTPS from day one</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>Required for microphone access and protects login/session data</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str"/>
+      <x:c r="D26" s="14" t="str"/>
+      <x:c r="E26" s="14" t="str"/>
+      <x:c r="F26" s="14" t="str"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="14" t="str">
+        <x:v>Keep founder-led support/moderation</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>Preserves cash until usage and safety workload are proven</x:v>
+      </x:c>
+      <x:c r="C27" s="14" t="str"/>
+      <x:c r="D27" s="14" t="str"/>
+      <x:c r="E27" s="14" t="str"/>
+      <x:c r="F27" s="14" t="str"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="14" t="str">
+        <x:v>Review usage monthly</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>Upgrade only when measured traffic, storage or incidents justify it</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str"/>
+      <x:c r="D28" s="14" t="str"/>
+      <x:c r="E28" s="14" t="str"/>
+      <x:c r="F28" s="14" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>Keep 3 months runway</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>Recommended cash reserve: 3 × average monthly startup burn</x:v>
+      </x:c>
+      <x:c r="C29" t="str"/>
+      <x:c r="D29" t="str"/>
+      <x:c r="E29" t="str"/>
+      <x:c r="F29" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A23:F23"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
model fixed seven lakh startup budget
</commit_message>
<xml_diff>
--- a/KNOMO_Worldwide_Tech_and_Costs.xlsx
+++ b/KNOMO_Worldwide_Tech_and_Costs.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive overview" sheetId="1" r:id="Rc388a1264da04478"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech stack" sheetId="2" r:id="R36a3277466ea4593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly costs" sheetId="3" r:id="Rd510773e0ab94cef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch checklist" sheetId="4" r:id="R82c806b1ae10481a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup year" sheetId="5" r:id="R3b6a51d2982e4db5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup year - leaner" sheetId="6" r:id="Rb115121a755345ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive overview" sheetId="1" r:id="R49b8fe69bdf142f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech stack" sheetId="2" r:id="Refdc8aa600c34f08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly costs" sheetId="3" r:id="R639499b9f3074289"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch checklist" sheetId="4" r:id="R2c4d50aee9354bb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup year" sheetId="5" r:id="R7ba43adaab82454c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Startup year - leaner" sheetId="6" r:id="R51e5932736984825"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="₹7 lakh startup plan" sheetId="7" r:id="R0bc67a4ab42342d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -83,7 +84,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -170,6 +171,31 @@
         <x:fgColor rgb="FF8E3B52"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF29353C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDFEBF6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF44576D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFAAC7D8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF8E3B52"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -191,7 +217,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="72">
+  <x:cellXfs count="89">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -310,6 +336,31 @@
     <x:xf numFmtId="200" fontId="4" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="3" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="3" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -2992,4 +3043,551 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="34" customHeight="1">
+      <x:c r="A1" s="74" t="str">
+        <x:v>KNOMO ₹7 lakh startup-year budget</x:v>
+      </x:c>
+      <x:c r="B1" s="74"/>
+      <x:c r="C1" s="74"/>
+      <x:c r="D1" s="74"/>
+      <x:c r="E1" s="74"/>
+      <x:c r="F1" s="74"/>
+      <x:c r="G1" s="74"/>
+      <x:c r="H1" s="74"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="77" t="str">
+        <x:v>Assumes a bootstrapped first year: founders cover product/engineering, use free tiers until usage proves demand, and pay only for production reliability and media. All amounts are INR (₹).</x:v>
+      </x:c>
+      <x:c r="B2" s="77"/>
+      <x:c r="C2" s="77"/>
+      <x:c r="D2" s="77"/>
+      <x:c r="E2" s="77"/>
+      <x:c r="F2" s="77"/>
+      <x:c r="G2" s="77"/>
+      <x:c r="H2" s="77"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="81" t="str">
+        <x:v>Budget line</x:v>
+      </x:c>
+      <x:c r="B4" s="81" t="str">
+        <x:v>Monthly ₹</x:v>
+      </x:c>
+      <x:c r="C4" s="81" t="str">
+        <x:v>Annual ₹</x:v>
+      </x:c>
+      <x:c r="D4" s="81" t="str">
+        <x:v>Type</x:v>
+      </x:c>
+      <x:c r="E4" s="81" t="str">
+        <x:v>Startup assumption</x:v>
+      </x:c>
+      <x:c r="F4" s="81" t="str">
+        <x:v>Trigger to upgrade</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="14" t="str">
+        <x:v>Domain + DNS + email</x:v>
+      </x:c>
+      <x:c r="B5" s="20" t="n">
+        <x:v>900</x:v>
+      </x:c>
+      <x:c r="C5" s="20" t="n">
+        <x:f>IF(D5="One-time",B5,B5*12)</x:f>
+        <x:v>10800</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E5" s="14" t="str">
+        <x:v>One domain and free/low-volume email tier</x:v>
+      </x:c>
+      <x:c r="F5" s="14" t="str">
+        <x:v>Upgrade when email volume or team grows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="14" t="str">
+        <x:v>Frontend hosting/CDN</x:v>
+      </x:c>
+      <x:c r="B6" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C6" s="20" t="n">
+        <x:f>IF(D6="One-time",B6,B6*12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E6" s="14" t="str">
+        <x:v>Free static hosting/CDN tier</x:v>
+      </x:c>
+      <x:c r="F6" s="14" t="str">
+        <x:v>Paid tier after bandwidth/build limits</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="14" t="str">
+        <x:v>API hosting</x:v>
+      </x:c>
+      <x:c r="B7" s="20" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="C7" s="20" t="n">
+        <x:f>IF(D7="One-time",B7,B7*12)</x:f>
+        <x:v>12000</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E7" s="14" t="str">
+        <x:v>Small production API tier; founders accept limited capacity</x:v>
+      </x:c>
+      <x:c r="F7" s="14" t="str">
+        <x:v>Add a second instance after uptime/load target is missed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="14" t="str">
+        <x:v>Managed database</x:v>
+      </x:c>
+      <x:c r="B8" s="20" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="C8" s="20" t="n">
+        <x:f>IF(D8="One-time",B8,B8*12)</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="D8" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E8" s="14" t="str">
+        <x:v>Small managed Postgres/MySQL with backups</x:v>
+      </x:c>
+      <x:c r="F8" s="14" t="str">
+        <x:v>Upgrade for storage, HA or replicas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="14" t="str">
+        <x:v>Object storage</x:v>
+      </x:c>
+      <x:c r="B9" s="20" t="n">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="C9" s="20" t="n">
+        <x:f>IF(D9="One-time",B9,B9*12)</x:f>
+        <x:v>2400</x:v>
+      </x:c>
+      <x:c r="D9" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="str">
+        <x:v>Small R2/S3 bucket; delete abandoned media quickly</x:v>
+      </x:c>
+      <x:c r="F9" s="14" t="str">
+        <x:v>Add retention tiers after media library grows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="14" t="str">
+        <x:v>Video processing/delivery</x:v>
+      </x:c>
+      <x:c r="B10" s="20" t="n">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="C10" s="20" t="n">
+        <x:f>IF(D10="One-time",B10,B10*12)</x:f>
+        <x:v>18000</x:v>
+      </x:c>
+      <x:c r="D10" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E10" s="14" t="str">
+        <x:v>Strict duration, size and monthly upload caps</x:v>
+      </x:c>
+      <x:c r="F10" s="14" t="str">
+        <x:v>Add transcoding workers as creator activity grows</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="14" t="str">
+        <x:v>Realtime/cache/queue</x:v>
+      </x:c>
+      <x:c r="B11" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C11" s="20" t="n">
+        <x:f>IF(D11="One-time",B11,B11*12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D11" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E11" s="14" t="str">
+        <x:v>Start with DB polling; add Redis only when live traffic needs it</x:v>
+      </x:c>
+      <x:c r="F11" s="14" t="str">
+        <x:v>Introduce Redis/WebSockets at sustained concurrency</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="14" t="str">
+        <x:v>Monitoring/security</x:v>
+      </x:c>
+      <x:c r="B12" s="20" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="C12" s="20" t="n">
+        <x:f>IF(D12="One-time",B12,B12*12)</x:f>
+        <x:v>6000</x:v>
+      </x:c>
+      <x:c r="D12" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E12" s="14" t="str">
+        <x:v>Free monitoring, logs and basic WAF rules</x:v>
+      </x:c>
+      <x:c r="F12" s="14" t="str">
+        <x:v>Upgrade after incident volume or compliance need</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="14" t="str">
+        <x:v>Backups/DR</x:v>
+      </x:c>
+      <x:c r="B13" s="20" t="n">
+        <x:v>300</x:v>
+      </x:c>
+      <x:c r="C13" s="20" t="n">
+        <x:f>IF(D13="One-time",B13,B13*12)</x:f>
+        <x:v>3600</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="str">
+        <x:v>Automated DB backup plus monthly restore drill</x:v>
+      </x:c>
+      <x:c r="F13" s="14" t="str">
+        <x:v>Add cross-region copies before larger launch</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="14" t="str">
+        <x:v>Support/moderation tools</x:v>
+      </x:c>
+      <x:c r="B14" s="20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C14" s="20" t="n">
+        <x:f>IF(D14="One-time",B14,B14*12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E14" s="14" t="str">
+        <x:v>Founder-led support and moderation using free tools</x:v>
+      </x:c>
+      <x:c r="F14" s="14" t="str">
+        <x:v>Hire part-time support after response SLA slips</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="14" t="str">
+        <x:v>Founder/contractor cash budget</x:v>
+      </x:c>
+      <x:c r="B15" s="20" t="n">
+        <x:v>5000</x:v>
+      </x:c>
+      <x:c r="C15" s="20" t="n">
+        <x:f>IF(D15="One-time",B15,B15*12)</x:f>
+        <x:v>60000</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="str">
+        <x:v>No planned contractor spend; small emergency allowance</x:v>
+      </x:c>
+      <x:c r="F15" s="14" t="str">
+        <x:v>Increase after revenue/funding milestone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="14" t="str">
+        <x:v>Product experiments + analytics</x:v>
+      </x:c>
+      <x:c r="B16" s="20" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="C16" s="20" t="n">
+        <x:f>IF(D16="One-time",B16,B16*12)</x:f>
+        <x:v>180000</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="str">
+        <x:v>Small budget for user research, analytics and UX tests</x:v>
+      </x:c>
+      <x:c r="F16" s="14" t="str">
+        <x:v>Increase after retention is proven</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="14" t="str">
+        <x:v>Creator/community launch budget</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="n">
+        <x:v>10000</x:v>
+      </x:c>
+      <x:c r="C17" s="20" t="n">
+        <x:f>IF(D17="One-time",B17,B17*12)</x:f>
+        <x:v>120000</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>Recurring</x:v>
+      </x:c>
+      <x:c r="E17" s="14" t="str">
+        <x:v>Small creator incentives and campus/community pilots</x:v>
+      </x:c>
+      <x:c r="F17" s="14" t="str">
+        <x:v>Increase only after activation is measurable</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="14" t="str">
+        <x:v>Company/legal/privacy setup</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="C18" s="20" t="n">
+        <x:f>IF(D18="One-time",B18,B18*12)</x:f>
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E18" s="14" t="str">
+        <x:v>Use templates plus one focused professional review</x:v>
+      </x:c>
+      <x:c r="F18" s="14" t="str">
+        <x:v>Repeat only for major jurisdictions or fundraising</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="14" t="str">
+        <x:v>Production migration + launch hardening</x:v>
+      </x:c>
+      <x:c r="B19" s="20" t="n">
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="C19" s="20" t="n">
+        <x:f>IF(D19="One-time",B19,B19*12)</x:f>
+        <x:v>25000</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E19" s="14" t="str">
+        <x:v>DIY migration, HTTPS, CI/CD and storage setup</x:v>
+      </x:c>
+      <x:c r="F19" s="14" t="str">
+        <x:v>Repeat for major architecture change</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="14" t="str">
+        <x:v>Security/load testing</x:v>
+      </x:c>
+      <x:c r="B20" s="20" t="n">
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="C20" s="20" t="n">
+        <x:f>IF(D20="One-time",B20,B20*12)</x:f>
+        <x:v>15000</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E20" s="14" t="str">
+        <x:v>Basic checklist and low-cost test before promotion</x:v>
+      </x:c>
+      <x:c r="F20" s="14" t="str">
+        <x:v>Repeat before major scale events</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="14" t="str">
+        <x:v>Unallocated runway reserve</x:v>
+      </x:c>
+      <x:c r="B21" s="20" t="n">
+        <x:v>204200</x:v>
+      </x:c>
+      <x:c r="C21" s="20" t="n">
+        <x:f>IF(D21="One-time",B21,B21*12)</x:f>
+        <x:v>204200</x:v>
+      </x:c>
+      <x:c r="D21" s="14" t="str">
+        <x:v>One-time</x:v>
+      </x:c>
+      <x:c r="E21" s="14" t="str">
+        <x:v>Held as cash buffer; do not spend without a measured trigger</x:v>
+      </x:c>
+      <x:c r="F21" s="14" t="str">
+        <x:v>Release only after monthly review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="83" t="str">
+        <x:v>Startup recurring subtotal</x:v>
+      </x:c>
+      <x:c r="B22" s="86" t="n">
+        <x:f>SUM(B5:B21)</x:f>
+        <x:v>305100</x:v>
+      </x:c>
+      <x:c r="C22" s="86" t="n">
+        <x:f>SUM(C5:C21)</x:f>
+        <x:v>700000</x:v>
+      </x:c>
+      <x:c r="D22" s="83" t="str"/>
+      <x:c r="E22" s="83" t="str"/>
+      <x:c r="F22" s="83" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="83" t="str">
+        <x:v>One-time launch subtotal</x:v>
+      </x:c>
+      <x:c r="B23" s="86"/>
+      <x:c r="C23" s="86" t="n">
+        <x:f>SUMIF(D5:D21,"One-time",C5:C21)</x:f>
+        <x:v>269200</x:v>
+      </x:c>
+      <x:c r="D23" s="83" t="str"/>
+      <x:c r="E23" s="83" t="str"/>
+      <x:c r="F23" s="83" t="str"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="85" t="str">
+        <x:v>Total first-year startup cash need</x:v>
+      </x:c>
+      <x:c r="B24" s="87"/>
+      <x:c r="C24" s="87" t="n">
+        <x:f>C22+C23</x:f>
+        <x:v>969200</x:v>
+      </x:c>
+      <x:c r="D24" s="85" t="str"/>
+      <x:c r="E24" s="85" t="str"/>
+      <x:c r="F24" s="85" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="83" t="str">
+        <x:v>Startup operating rules</x:v>
+      </x:c>
+      <x:c r="B26" s="83"/>
+      <x:c r="C26" s="83"/>
+      <x:c r="D26" s="83"/>
+      <x:c r="E26" s="83"/>
+      <x:c r="F26" s="83"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="81" t="str">
+        <x:v>Rule</x:v>
+      </x:c>
+      <x:c r="B27" s="81" t="str">
+        <x:v>Why it matters</x:v>
+      </x:c>
+      <x:c r="C27" s="81" t="str"/>
+      <x:c r="D27" s="81" t="str"/>
+      <x:c r="E27" s="81" t="str"/>
+      <x:c r="F27" s="81" t="str"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="14" t="str">
+        <x:v>Cap video duration and file size</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>Video is the largest variable cost; caps prevent surprise bills</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str"/>
+      <x:c r="D28" s="14" t="str"/>
+      <x:c r="E28" s="14" t="str"/>
+      <x:c r="F28" s="14" t="str"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="14" t="str">
+        <x:v>Use HTTPS from day one</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>Required for microphone access and protects login/session data</x:v>
+      </x:c>
+      <x:c r="C29" s="14" t="str"/>
+      <x:c r="D29" s="14" t="str"/>
+      <x:c r="E29" s="14" t="str"/>
+      <x:c r="F29" s="14" t="str"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="14" t="str">
+        <x:v>Keep founder-led support/moderation</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>Preserves cash until usage and safety workload are proven</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str"/>
+      <x:c r="D30" s="14" t="str"/>
+      <x:c r="E30" s="14" t="str"/>
+      <x:c r="F30" s="14" t="str"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="14" t="str">
+        <x:v>Review usage monthly</x:v>
+      </x:c>
+      <x:c r="B31" s="14" t="str">
+        <x:v>Upgrade only when measured traffic, storage or incidents justify it</x:v>
+      </x:c>
+      <x:c r="C31" s="14" t="str"/>
+      <x:c r="D31" s="14" t="str"/>
+      <x:c r="E31" s="14" t="str"/>
+      <x:c r="F31" s="14" t="str"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>Keep 3 months runway</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>Recommended cash reserve: 3 × average monthly startup burn</x:v>
+      </x:c>
+      <x:c r="C32" t="str"/>
+      <x:c r="D32" t="str"/>
+      <x:c r="E32" t="str"/>
+      <x:c r="F32" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A26:F26"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>